<commit_message>
Updated EDI files and converted files for the release
</commit_message>
<xml_diff>
--- a/converted_files/834/834-all-fields.xlsx
+++ b/converted_files/834/834-all-fields.xlsx
@@ -2222,7 +2222,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>6976904ee9a75feb648555f5</t>
+          <t>69efef04ad4799caa7f5a7c4</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0001</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="AH2" s="3" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AI2" s="3" t="inlineStr">
@@ -2580,7 +2580,7 @@
       </c>
       <c r="CQ2" s="3" t="inlineStr">
         <is>
-          <t>SalaryGrade</t>
+          <t>Grade</t>
         </is>
       </c>
       <c r="CR2" s="3" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="EF2" s="3" t="inlineStr">
         <is>
-          <t>HOME_PHONE</t>
+          <t>PHONE</t>
         </is>
       </c>
       <c r="EG2" s="3" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="EH2" s="3" t="inlineStr">
         <is>
-          <t>WORK_PHONE</t>
+          <t>PHONE</t>
         </is>
       </c>
       <c r="EI2" s="3" t="inlineStr">
@@ -2789,7 +2789,7 @@
       </c>
       <c r="FD2" s="3" t="inlineStr">
         <is>
-          <t>HOME_PHONE</t>
+          <t>PHONE</t>
         </is>
       </c>
       <c r="FE2" s="3" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="FF2" s="3" t="inlineStr">
         <is>
-          <t>WORK_PHONE</t>
+          <t>PHONE</t>
         </is>
       </c>
       <c r="FG2" s="3" t="inlineStr">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="NO2" s="3" t="inlineStr">
         <is>
-          <t>HOME_PHONE</t>
+          <t>PHONE</t>
         </is>
       </c>
       <c r="NP2" s="3" t="inlineStr">
@@ -3503,7 +3503,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>6976904ee9a75feb648555f5</t>
+          <t>69efef04ad4799caa7f5a7c4</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -3513,7 +3513,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0001</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -3648,7 +3648,7 @@
       </c>
       <c r="AH3" s="3" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AI3" s="3" t="inlineStr">
@@ -3861,7 +3861,7 @@
       </c>
       <c r="CQ3" s="3" t="inlineStr">
         <is>
-          <t>SalaryGrade</t>
+          <t>Grade</t>
         </is>
       </c>
       <c r="CR3" s="3" t="inlineStr">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="EF3" s="3" t="inlineStr">
         <is>
-          <t>HOME_PHONE</t>
+          <t>PHONE</t>
         </is>
       </c>
       <c r="EG3" s="3" t="inlineStr">
@@ -4020,7 +4020,7 @@
       </c>
       <c r="EH3" s="3" t="inlineStr">
         <is>
-          <t>WORK_PHONE</t>
+          <t>PHONE</t>
         </is>
       </c>
       <c r="EI3" s="3" t="inlineStr">
@@ -4070,7 +4070,7 @@
       </c>
       <c r="FD3" s="3" t="inlineStr">
         <is>
-          <t>HOME_PHONE</t>
+          <t>PHONE</t>
         </is>
       </c>
       <c r="FE3" s="3" t="inlineStr">
@@ -4080,7 +4080,7 @@
       </c>
       <c r="FF3" s="3" t="inlineStr">
         <is>
-          <t>WORK_PHONE</t>
+          <t>PHONE</t>
         </is>
       </c>
       <c r="FG3" s="3" t="inlineStr">
@@ -4574,7 +4574,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>6976904ee9a75feb648555f6</t>
+          <t>69efef04ad4799caa7f5a7c5</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -4584,7 +4584,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0001</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -5231,7 +5231,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>6976904ee9a75feb648555f7</t>
+          <t>69efef04ad4799caa7f5a7c6</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -5241,7 +5241,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0002</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -5272,7 +5272,7 @@
       <c r="M5"/>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>MasterPolicyNumbe2</t>
+          <t>MasterPolicyNumber2</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
@@ -5332,7 +5332,7 @@
       <c r="AG5"/>
       <c r="AH5" s="3" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>9</t>
         </is>
       </c>
       <c r="AI5" s="3" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="AJ5" s="3" t="inlineStr">
         <is>
-          <t>ST</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AK5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Added EDI samples with validation issues; regenerated examples
</commit_message>
<xml_diff>
--- a/converted_files/834/834-all-fields.xlsx
+++ b/converted_files/834/834-all-fields.xlsx
@@ -2222,7 +2222,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>69e82c67836d7d05c9a01977</t>
+          <t>6a04c9e830180e9da6b3fdc8</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -3503,7 +3503,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>69e82c67836d7d05c9a01977</t>
+          <t>6a04c9e830180e9da6b3fdc8</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -4574,7 +4574,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>69e82c67836d7d05c9a01978</t>
+          <t>6a04c9e830180e9da6b3fdc9</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -5231,7 +5231,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>69e82c67836d7d05c9a01979</t>
+          <t>6a04c9e830180e9da6b3fdca</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Updated all EDI generated files to include new fields from 2.14.10
</commit_message>
<xml_diff>
--- a/converted_files/834/834-all-fields.xlsx
+++ b/converted_files/834/834-all-fields.xlsx
@@ -2222,7 +2222,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>6a04c9e830180e9da6b3fdc8</t>
+          <t>6a04cc591ef26d534baf0403</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -3503,7 +3503,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>6a04c9e830180e9da6b3fdc8</t>
+          <t>6a04cc591ef26d534baf0403</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -4574,7 +4574,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>6a04c9e830180e9da6b3fdc9</t>
+          <t>6a04cc591ef26d534baf0404</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -5231,7 +5231,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>6a04c9e830180e9da6b3fdca</t>
+          <t>6a04cc591ef26d534baf0405</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Updated converted and generated files examples
</commit_message>
<xml_diff>
--- a/converted_files/834/834-all-fields.xlsx
+++ b/converted_files/834/834-all-fields.xlsx
@@ -2222,7 +2222,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>6a04cc591ef26d534baf0403</t>
+          <t>6a32cb6297613a0e499056c7</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -3503,7 +3503,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>6a04cc591ef26d534baf0403</t>
+          <t>6a32cb6297613a0e499056c7</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -4574,7 +4574,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>6a04cc591ef26d534baf0404</t>
+          <t>6a32cb6297613a0e499056c8</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -5231,7 +5231,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>6a04cc591ef26d534baf0405</t>
+          <t>6a32cb6297613a0e499056c9</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">

</xml_diff>